<commit_message>
Add points for cz84ih3b6irraa24kj6kvtz4k_playerlog
</commit_message>
<xml_diff>
--- a/bnc-streamlit-app/data/points/cz84ih3b6irraa24kj6kvtz4k_playerlog.xlsx
+++ b/bnc-streamlit-app/data/points/cz84ih3b6irraa24kj6kvtz4k_playerlog.xlsx
@@ -1969,7 +1969,7 @@
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>0.50835284</v>
+        <v>0.5052774200000001</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
@@ -2158,7 +2158,7 @@
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>-0.18</t>
+          <t>-0.17</t>
         </is>
       </c>
       <c r="AK9" t="n">
@@ -2286,7 +2286,11 @@
       <c r="N10" t="n">
         <v>95</v>
       </c>
-      <c r="O10" t="inlineStr"/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
       <c r="P10" t="n">
         <v>0</v>
       </c>
@@ -2299,10 +2303,16 @@
         </is>
       </c>
       <c r="S10" t="n">
-        <v>95</v>
-      </c>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
+        <v>84.3</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
+      <c r="U10" t="n">
+        <v>10.7</v>
+      </c>
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr"/>
@@ -2337,15 +2347,15 @@
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>0.06619631000000002</v>
+        <v>0.07084671000000002</v>
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>-0.61</t>
+          <t>-0.60</t>
         </is>
       </c>
       <c r="AK10" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="AL10" t="n">
         <v>0</v>
@@ -2536,7 +2546,7 @@
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>-0.07</t>
+          <t>-0.06</t>
         </is>
       </c>
       <c r="AK11" t="n">
@@ -2914,11 +2924,11 @@
         </is>
       </c>
       <c r="AI13" t="n">
-        <v>0.27368628</v>
+        <v>0.26903588</v>
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>-0.40</t>
+          <t>-0.41</t>
         </is>
       </c>
       <c r="AK13" t="n">
@@ -3111,7 +3121,7 @@
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>0.22071922</v>
+        <v>0.2218108</v>
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
@@ -3249,7 +3259,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>LW</t>
+          <t>LW, RCM(2)</t>
         </is>
       </c>
       <c r="P15" t="n">
@@ -3272,10 +3282,16 @@
         </is>
       </c>
       <c r="U15" t="n">
-        <v>17</v>
-      </c>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
+        <v>6.3</v>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>RCM(2)</t>
+        </is>
+      </c>
+      <c r="W15" t="n">
+        <v>10.7</v>
+      </c>
       <c r="X15" t="inlineStr"/>
       <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="inlineStr"/>
@@ -3444,7 +3460,11 @@
       <c r="N16" t="n">
         <v>11</v>
       </c>
-      <c r="O16" t="inlineStr"/>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
       <c r="P16" t="n">
         <v>84</v>
       </c>
@@ -3457,10 +3477,16 @@
         </is>
       </c>
       <c r="S16" t="n">
-        <v>11</v>
-      </c>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
+        <v>0.3</v>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="U16" t="n">
+        <v>10.7</v>
+      </c>
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
       <c r="X16" t="inlineStr"/>
@@ -3503,7 +3529,7 @@
         </is>
       </c>
       <c r="AK16" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AL16" t="n">
         <v>84</v>
@@ -3633,7 +3659,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>AM, CF</t>
         </is>
       </c>
       <c r="P17" t="n">
@@ -3656,10 +3682,16 @@
         </is>
       </c>
       <c r="U17" t="n">
-        <v>17</v>
-      </c>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
+        <v>6.3</v>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="W17" t="n">
+        <v>10.7</v>
+      </c>
       <c r="X17" t="inlineStr"/>
       <c r="Y17" t="inlineStr"/>
       <c r="Z17" t="inlineStr"/>
@@ -3692,7 +3724,7 @@
         </is>
       </c>
       <c r="AI17" t="n">
-        <v>0.05517638</v>
+        <v>0.05891353000000001</v>
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
@@ -5763,11 +5795,11 @@
         </is>
       </c>
       <c r="AI28" t="n">
-        <v>2.04695872</v>
+        <v>2.02515653</v>
       </c>
       <c r="AJ28" t="inlineStr">
         <is>
-          <t>+1.37</t>
+          <t>+1.35</t>
         </is>
       </c>
       <c r="AK28" t="n">
@@ -5792,7 +5824,7 @@
         <v>4</v>
       </c>
       <c r="AR28" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AS28" t="n">
         <v>0</v>
@@ -5833,13 +5865,13 @@
         </is>
       </c>
       <c r="BE28" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="BF28" t="n">
         <v>10</v>
       </c>
       <c r="BG28" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29">
@@ -6342,7 +6374,7 @@
       </c>
       <c r="AJ31" t="inlineStr">
         <is>
-          <t>-0.28</t>
+          <t>-0.27</t>
         </is>
       </c>
       <c r="AK31" t="n">
@@ -6525,11 +6557,11 @@
         </is>
       </c>
       <c r="AI32" t="n">
-        <v>0.85304212</v>
+        <v>0.86552556</v>
       </c>
       <c r="AJ32" t="inlineStr">
         <is>
-          <t>+0.18</t>
+          <t>+0.19</t>
         </is>
       </c>
       <c r="AK32" t="n">
@@ -6554,7 +6586,7 @@
         <v>0</v>
       </c>
       <c r="AR32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AS32" t="n">
         <v>1</v>
@@ -6722,11 +6754,11 @@
         </is>
       </c>
       <c r="AI33" t="n">
-        <v>0.36525078</v>
+        <v>0.35251578</v>
       </c>
       <c r="AJ33" t="inlineStr">
         <is>
-          <t>-0.31</t>
+          <t>-0.32</t>
         </is>
       </c>
       <c r="AK33" t="n">

</xml_diff>